<commit_message>
Add Marine Diesel overview PDF; refresh model thesis text
Five-page IC overview built in the fund-communications design theme
(Source Serif / Public Sans, deep-teal data palette, disclosure on every
page), branded Leviathan. Thesis Review text in the workbook updated to
match the final capital stack and synergy assumptions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZmF5WpT7AoC7xtqjtfCyZ
</commit_message>
<xml_diff>
--- a/models/Leviathan_Infra_RollUp_MarineDiesel_Model_v1.xlsx
+++ b/models/Leviathan_Infra_RollUp_MarineDiesel_Model_v1.xlsx
@@ -192,7 +192,7 @@
     <t xml:space="preserve">5x+ the $15M mandate. CIM never shows a capital stack.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hard $15M Leviathan cap. Stack: 2.25x senior + DDTL (40% of add-on EV) + seller notes (10-15%) + rollover (5-15%) + earnouts (10%) + retained FCF. Revolver only after cap is exhausted.</t>
+    <t xml:space="preserve">Hard $15M Leviathan cap. Stack: 2.25x senior + DDTL (35% of add-on EV) + seller notes (10-15%) + rollover (5-15%) + earnouts (10%) + a 25% minimum sponsor-equity slice per add-on + retained FCF. Revolver only after the cap is used up.</t>
   </si>
   <si>
     <t xml:space="preserve">Assumptions B-col capital block; Sources &amp; Uses</t>
@@ -207,7 +207,7 @@
     <t xml:space="preserve">Top of range unaffordable under the cap.</t>
   </si>
   <si>
-    <t xml:space="preserve">$10M revenue / 18% normalized margin (QoE haircut) / 5.25x. ~$2.4M Leviathan check at close leaves ~$12.6M for add-ons.</t>
+    <t xml:space="preserve">$10M revenue / 18% normalized margin (QoE haircut) / 5.25x. ~$3.0M Leviathan check at close leaves ~$12.0M for add-ons.</t>
   </si>
   <si>
     <t xml:space="preserve">plat_rev, plat_margin, plat_mult</t>
@@ -222,7 +222,7 @@
     <t xml:space="preserve">Owner-operated marine shops normalize to 12-18%. OEM parts GM is closer to 30-40%.</t>
   </si>
   <si>
-    <t xml:space="preserve">Platform 18% / add-ons 14% standalone + bottom-up synergies (~5.5 pts) less a real HQ cost line ($1.0M growing 8%).</t>
+    <t xml:space="preserve">Platform 18% / add-ons 14% standalone + bottom-up synergies (~6.0 pts) less a real HQ cost line ($1.0M growing 8%).</t>
   </si>
   <si>
     <t xml:space="preserve">Synergies tab part A; oh1</t>
@@ -237,7 +237,7 @@
     <t xml:space="preserve">Double-counts: overhead savings with no HQ cost; 85-95% utilization means technicians relocate seasonally.</t>
   </si>
   <si>
-    <t xml:space="preserve">Back-office +3 pts net; utilization 70% -&gt; 80% with 25% flow-through; procurement 10% on parts COGS.</t>
+    <t xml:space="preserve">Back-office +2 pts net; utilization 70% -&gt; 80% with 20% flow-through; procurement 10% on parts COGS; pricing/mix +0.75 pts.</t>
   </si>
   <si>
     <t xml:space="preserve">Synergies C5:D12</t>

</xml_diff>